<commit_message>
change text on the figure
</commit_message>
<xml_diff>
--- a/interface/detect/only_table/detection_table.xlsx
+++ b/interface/detect/only_table/detection_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yue\Desktop\newPeng\Peng1.0_GUI\interface\detect\only_table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868DCBCC-3F44-44A5-ACD1-1655813DFCB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E676E364-52F3-4782-9110-4AF56729629F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2380" yWindow="4450" windowWidth="25000" windowHeight="16430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3480" yWindow="4450" windowWidth="25000" windowHeight="16430" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -427,16 +427,16 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>141.34411686677191</v>
+        <v>140.9128656719823</v>
       </c>
       <c r="C2">
-        <v>168.50339387268389</v>
+        <v>168.37386877828061</v>
       </c>
       <c r="D2">
-        <v>168.726288754357</v>
+        <v>168.80392156862749</v>
       </c>
       <c r="E2">
-        <v>190.43845166024579</v>
+        <v>190.25697586727</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -444,16 +444,16 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>126.6541147292364</v>
+        <v>126.89278263202461</v>
       </c>
       <c r="C3">
-        <v>164.09129267357119</v>
+        <v>164.1629759129759</v>
       </c>
       <c r="D3">
-        <v>169.26831607211349</v>
+        <v>169.24805749805751</v>
       </c>
       <c r="E3">
-        <v>198.3084004602992</v>
+        <v>198.3982128982129</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -461,16 +461,16 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>144.29700761125491</v>
+        <v>144.54394736855491</v>
       </c>
       <c r="C4">
-        <v>169.390286377709</v>
+        <v>169.46445404556169</v>
       </c>
       <c r="D4">
-        <v>170.31985294117649</v>
+        <v>170.28711704634719</v>
       </c>
       <c r="E4">
-        <v>192.24922600619189</v>
+        <v>192.24862529457971</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -478,16 +478,16 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>138.23510061817589</v>
+        <v>138.13617719242481</v>
       </c>
       <c r="C5">
-        <v>167.56960950764011</v>
+        <v>167.53989813242791</v>
       </c>
       <c r="D5">
-        <v>173.84231748726651</v>
+        <v>173.86757215619701</v>
       </c>
       <c r="E5">
-        <v>199.14770797962649</v>
+        <v>199.1464346349745</v>
       </c>
     </row>
   </sheetData>

</xml_diff>